<commit_message>
Caso colombiano 18 nodos: red, generacion, demanda e hidraulicas
- Red equivalente de 18 subareas desde PARATEC (26 enlaces)
- Generadores agregados por subarea y fuente energetica
- Demanda nodal desde DemaOR con mapeo a subareas operativas
- Bloque hidraulico: 18 embalses + 4 bloques filo de agua
- Perfil solar horario desde metrica Gene de XM
- Formulacion TCSC por bloques discretos de compensacion

Estado: E0 infactible por interaccion entre Pmin hidraulico
y la restriccion V_T = V_init. Diagnostico en curso.
</commit_message>
<xml_diff>
--- a/01_Data/01_Raw/XM_API/inventario_metricas_xm.xlsx
+++ b/01_Data/01_Raw/XM_API/inventario_metricas_xm.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\API_XM-master_SINGIT\00_dalp\datos_xm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\01_Raw\XM_API\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3739D0CB-14B7-4C5F-B585-C20830A92715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08130163-77AC-4F81-A6EF-9F3FC9BC8B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4D1F358-1B09-4AC1-8F89-0B133C0C9CAC}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4D1F358-1B09-4AC1-8F89-0B133C0C9CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="inventario_metricas_xm" sheetId="1" r:id="rId1"/>
@@ -2087,7 +2087,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFDAF2D0"/>
+          <fgColor rgb="FFCAEDFB"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -6294,8 +6294,8 @@
         <v>332</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A134" s="4" t="s">
         <v>333</v>
       </c>
       <c r="B134" t="s">

</xml_diff>

<commit_message>
COL 18 + COL 110
- Se incluye compensación no solo capacitiva sino inductiva también
- Se modela sistema colombiano de 110 nodos
- IPOEL (Informe de planeamiento operativo eléctrico de mediano y largo plazo)
</commit_message>
<xml_diff>
--- a/01_Data/01_Raw/XM_API/inventario_metricas_xm.xlsx
+++ b/01_Data/01_Raw/XM_API/inventario_metricas_xm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\01_Raw\XM_API\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08130163-77AC-4F81-A6EF-9F3FC9BC8B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7EA6543-8ED3-45A1-BA60-5871B3B265D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4D1F358-1B09-4AC1-8F89-0B133C0C9CAC}"/>
+    <workbookView xWindow="22932" yWindow="780" windowWidth="23256" windowHeight="12456" xr2:uid="{E4D1F358-1B09-4AC1-8F89-0B133C0C9CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="inventario_metricas_xm" sheetId="1" r:id="rId1"/>
@@ -6845,8 +6845,8 @@
         <v>379</v>
       </c>
     </row>
-    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A153" s="4" t="s">
         <v>380</v>
       </c>
       <c r="B153" t="s">
@@ -6961,8 +6961,8 @@
         <v>392</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A157" s="4" t="s">
         <v>393</v>
       </c>
       <c r="B157" t="s">
@@ -6990,8 +6990,8 @@
         <v>382</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A158" s="4" t="s">
         <v>393</v>
       </c>
       <c r="B158" t="s">

</xml_diff>